<commit_message>
fix(gist): make the LinkML converter's output deterministic
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/gist.xlsx
+++ b/project/excel/gist.xlsx
@@ -7,102 +7,102 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="GeoPoint" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Specification" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Event" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ElectronicAddress" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Tag" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TemporalRelation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Landmark" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Address" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ReferenceValue" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Function" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ContemporaryEvent" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Person" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="PhysicalAddress" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="UnitOfMeasure" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="GeoRegion" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Agreement" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Composite" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Account" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Address" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="AddressUsageType" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Agreement" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Aspect" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Assignment" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Behavior" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Building" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="BundledCatalogItem" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="CatalogItem" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Category" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Collection" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Commitment" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Component" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Composite" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="ContemporaryEvent" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Content" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="ContentExpression" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="OrderedMember" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Commitment" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Text" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="MediaType" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="IntergovernmentalOrganization" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Task" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Component" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="ContingentObligation" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Language" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="PhysicalActionType" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Message" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="PhysicalAddressType" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="ContingentEvent" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="ContingentObligation" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Contract" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="ContractTerm" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="ControlledVocabulary" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="CountryGeoRegion" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="CountryGovernment" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="DegreeOfCommitment" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Determination" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Discipline" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="ElectronicAddress" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="ElectronicAddressType" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="Equipment" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="Transaction" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="Network" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="Assignment" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="HistoricalEvent" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="DegreeOfCommitment" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="TimeInterval" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="Magnitude" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="ControlledVocabulary" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="LivingThing" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="UnitGroup" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="System" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="Behavior" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="ID" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="ScheduledEvent" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="Building" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="ScheduledTask" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="Permission" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="ServiceSpecification" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="NetworkNode" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="Organization" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="ContractTerm" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="OrderedCollection" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="SubCountryGovernment" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="AddressUsageType" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="TaskTemplate" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="CatalogItem" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="PhysicalSubstance" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="RenderedContent" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="Collection" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="EquipmentType" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="EventSpecification" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="Account" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="Aspect" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="Requirement" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="KnowledgeConcept" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="IntellectualProperty" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="Determination" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="ElectronicAddressType" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="Medium" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="GovernmentOrganization" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="GeneralMediaType" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="PhysicalIdentifiableItem" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="GeoVolume" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="Contract" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="Category" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="Restriction" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="FormattedContent" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="Intention" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet name="Project" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet name="Content" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet name="ProductCategory" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet name="ProductSpecification" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet name="CountryGovernment" sheetId="84" state="visible" r:id="rId84"/>
-    <sheet name="BundledCatalogItem" sheetId="85" state="visible" r:id="rId85"/>
-    <sheet name="Offer" sheetId="86" state="visible" r:id="rId86"/>
-    <sheet name="NetworkLink" sheetId="87" state="visible" r:id="rId87"/>
-    <sheet name="Discipline" sheetId="88" state="visible" r:id="rId88"/>
-    <sheet name="Template" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet name="PhysicalEvent" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet name="GovernedGeoRegion" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet name="GeoLocation" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet name="GeoRoute" sheetId="93" state="visible" r:id="rId93"/>
-    <sheet name="CountryGeoRegion" sheetId="94" state="visible" r:id="rId94"/>
-    <sheet name="ContingentEvent" sheetId="95" state="visible" r:id="rId95"/>
-    <sheet name="SchemaMetaData" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet name="EquipmentType" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Event" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="EventSpecification" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="FormattedContent" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="Function" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="GeneralMediaType" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="GeoLocation" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="GeoPoint" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="GeoRegion" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="GeoRoute" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="GeoVolume" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="GovernedGeoRegion" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="GovernmentOrganization" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="HistoricalEvent" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="ID" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="IntellectualProperty" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="Intention" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="IntergovernmentalOrganization" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="KnowledgeConcept" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="Landmark" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="Language" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="LivingThing" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="Magnitude" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="MediaType" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="Medium" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="Message" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="Network" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="NetworkLink" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="NetworkNode" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="Offer" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="OrderedCollection" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="OrderedMember" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="Organization" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="Permission" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="Person" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="PhysicalActionType" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="PhysicalAddress" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="PhysicalAddressType" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="PhysicalEvent" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="PhysicalIdentifiableItem" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="PhysicalSubstance" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="ProductCategory" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="ProductSpecification" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="Project" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="ReferenceValue" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="RenderedContent" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="Requirement" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="Restriction" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="ScheduledEvent" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="ScheduledTask" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="SchemaMetaData" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="ServiceSpecification" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet name="Specification" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet name="SubCountryGovernment" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet name="System" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet name="Tag" sheetId="87" state="visible" r:id="rId87"/>
+    <sheet name="Task" sheetId="88" state="visible" r:id="rId88"/>
+    <sheet name="TaskTemplate" sheetId="89" state="visible" r:id="rId89"/>
+    <sheet name="Template" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet name="TemporalRelation" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet name="Text" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet name="TimeInterval" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet name="Transaction" sheetId="94" state="visible" r:id="rId94"/>
+    <sheet name="UnitGroup" sheetId="95" state="visible" r:id="rId95"/>
+    <sheet name="UnitOfMeasure" sheetId="96" state="visible" r:id="rId96"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix(converter): range unranged object properties over Any, not string
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/gist.xlsx
+++ b/project/excel/gist.xlsx
@@ -103,6 +103,7 @@
     <sheet name="Transaction" sheetId="94" state="visible" r:id="rId94"/>
     <sheet name="UnitGroup" sheetId="95" state="visible" r:id="rId95"/>
     <sheet name="UnitOfMeasure" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet name="Any" sheetId="97" state="visible" r:id="rId97"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2996,4 +2997,17 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet97.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(converter): range unranged object properties over Any, not string (#14)
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/gist.xlsx
+++ b/project/excel/gist.xlsx
@@ -103,6 +103,7 @@
     <sheet name="Transaction" sheetId="94" state="visible" r:id="rId94"/>
     <sheet name="UnitGroup" sheetId="95" state="visible" r:id="rId95"/>
     <sheet name="UnitOfMeasure" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet name="Any" sheetId="97" state="visible" r:id="rId97"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2996,4 +2997,17 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet97.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>